<commit_message>
Sync full ES2M main snapshot
</commit_message>
<xml_diff>
--- a/docs/martial_arts/武功強度設定表.xlsx
+++ b/docs/martial_arts/武功強度設定表.xlsx
@@ -836,7 +836,7 @@
         <v>30</v>
       </c>
       <c r="J2" s="8" t="n">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="K2" s="8" t="n">
         <v>10</v>
@@ -10831,7 +10831,7 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>給「武學之道」=（新等級 − 減數）× 係數。（龍圖心經：起始 51、減數 41、係數 10；三門刀法定案：起始 30、減數 11、係數 10）</t>
+          <t>給「武學之道」=（新等級 − 減數）× 係數。（龍圖心經：起始 51、減數 41、係數 10；三門刀法定案：起始 30、減數 29、係數 10）</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">

</xml_diff>